<commit_message>
Add Guerrero's Ex4A and Update Guerrero Excel
</commit_message>
<xml_diff>
--- a/Guerrero_Ex3A_tables.xlsx
+++ b/Guerrero_Ex3A_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sguer\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36514287-2D1B-47DC-8BCA-0C44BD61F019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7513C413-B205-48D2-A54A-77FF9E257298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" firstSheet="3" activeTab="4" xr2:uid="{95D1C2D3-DDB1-4C63-A4EA-1389BC982B33}"/>
+    <workbookView xWindow="1132" yWindow="293" windowWidth="20025" windowHeight="12285" activeTab="3" xr2:uid="{95D1C2D3-DDB1-4C63-A4EA-1389BC982B33}"/>
   </bookViews>
   <sheets>
     <sheet name="Clients" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="77">
   <si>
     <t>1st table:</t>
   </si>
@@ -168,9 +168,6 @@
     <t>Price</t>
   </si>
   <si>
-    <t>PaymentConfirmation</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -308,12 +305,79 @@
   <si>
     <t>Notes</t>
   </si>
+  <si>
+    <t>ClientsID</t>
+  </si>
+  <si>
+    <t>Oscar Ramos</t>
+  </si>
+  <si>
+    <t>551-300-9976</t>
+  </si>
+  <si>
+    <t>214 60th St</t>
+  </si>
+  <si>
+    <t>West New York</t>
+  </si>
+  <si>
+    <t>NJ</t>
+  </si>
+  <si>
+    <t>oscarsuriano14@gmail.com</t>
+  </si>
+  <si>
+    <t>DogID</t>
+  </si>
+  <si>
+    <t>ClientID</t>
+  </si>
+  <si>
+    <t>Axel</t>
+  </si>
+  <si>
+    <t>Siberian Husky</t>
+  </si>
+  <si>
+    <t>Axel is very friendly with children!</t>
+  </si>
+  <si>
+    <t>AppointmentID</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>PaymentID</t>
+  </si>
+  <si>
+    <t>2016-02-12</t>
+  </si>
+  <si>
+    <t>2026-02-12</t>
+  </si>
+  <si>
+    <t>Debit</t>
+  </si>
+  <si>
+    <t>LogID</t>
+  </si>
+  <si>
+    <t>Axel's collar is too large for his neck and accidentally unclasped, recommend a vest collar</t>
+  </si>
+  <si>
+    <t>PaymentStatus</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -336,8 +400,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -360,6 +439,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -387,10 +478,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -404,14 +496,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -744,23 +872,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2398A5B-FBD8-4D77-92F2-DFF8B3618123}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.19921875" customWidth="1"/>
     <col min="2" max="2" width="17.73046875" customWidth="1"/>
     <col min="3" max="3" width="31.1328125" customWidth="1"/>
-    <col min="4" max="4" width="14.53125" customWidth="1"/>
+    <col min="4" max="4" width="26.59765625" customWidth="1"/>
     <col min="5" max="5" width="18.59765625" customWidth="1"/>
     <col min="6" max="6" width="18.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -768,7 +896,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>26</v>
       </c>
@@ -776,15 +904,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="5" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A4" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
@@ -792,7 +920,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
@@ -800,7 +928,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
@@ -808,7 +936,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
@@ -816,7 +944,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
         <v>9</v>
       </c>
@@ -824,7 +952,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
         <v>10</v>
       </c>
@@ -832,26 +960,83 @@
         <v>18</v>
       </c>
     </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A12" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A13" s="7">
+        <v>1</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>61</v>
+      </c>
+      <c r="H13">
+        <v>70930</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D13" r:id="rId1" xr:uid="{5E78E9F1-AF7E-4D3A-96C0-CEC93132B1C8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82763257-DCF9-4E9D-861B-824F69A28B27}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.3984375" customWidth="1"/>
     <col min="2" max="2" width="15.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="5" width="13.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>19</v>
       </c>
@@ -859,23 +1044,23 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="6" t="s">
-        <v>46</v>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" s="5" t="s">
+        <v>45</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
         <v>20</v>
       </c>
@@ -883,7 +1068,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
@@ -891,7 +1076,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>22</v>
       </c>
@@ -899,12 +1084,52 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
         <v>24</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A10" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="A11" s="13">
+        <v>1</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="13">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -914,19 +1139,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25C0138B-8C0C-4F85-9A62-5C9017072CA0}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.796875" customWidth="1"/>
     <col min="2" max="2" width="15.86328125" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>27</v>
       </c>
@@ -934,39 +1161,39 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="6" t="s">
-        <v>46</v>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A4" s="5" t="s">
+        <v>45</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" s="6" t="s">
-        <v>47</v>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A5" s="5" t="s">
+        <v>46</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>28</v>
       </c>
@@ -974,7 +1201,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
         <v>31</v>
       </c>
@@ -982,12 +1209,58 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A11" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A12" s="7">
+        <v>1</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="17">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="D12" s="19">
+        <v>60</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -997,19 +1270,22 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C10CFC92-4B73-4EE5-AA04-7FD2CE0058EB}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="18.59765625" customWidth="1"/>
     <col min="2" max="2" width="13.59765625" customWidth="1"/>
+    <col min="3" max="3" width="15.1328125" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" customWidth="1"/>
+    <col min="6" max="6" width="13.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>34</v>
       </c>
@@ -1017,23 +1293,23 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="6" t="s">
-        <v>45</v>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" s="5" t="s">
+        <v>44</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
         <v>35</v>
       </c>
@@ -1041,28 +1317,68 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
         <v>36</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
         <v>37</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>42</v>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A10" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A11" s="7">
+        <v>1</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="21">
+        <v>25.99</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1072,72 +1388,116 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09B45A92-2EF5-4550-AC98-59AB90B700D0}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="19.3984375" customWidth="1"/>
     <col min="2" max="2" width="17.19921875" customWidth="1"/>
+    <col min="3" max="3" width="16.46484375" customWidth="1"/>
+    <col min="4" max="4" width="13.86328125" customWidth="1"/>
+    <col min="5" max="5" width="15.46484375" customWidth="1"/>
+    <col min="6" max="6" width="13.9296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
         <v>49</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A2" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="6" t="s">
-        <v>45</v>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" s="5" t="s">
+        <v>44</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" s="6" t="s">
-        <v>47</v>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A5" s="5" t="s">
+        <v>46</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B7" s="4" t="s">
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A8" s="4" t="s">
         <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A8" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A10" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="A11" s="22">
+        <v>1</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="23">
+        <v>3.5</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="25">
+        <v>1</v>
+      </c>
+      <c r="F11" s="25">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>